<commit_message>
Daily NAV update 2026-04-08
</commit_message>
<xml_diff>
--- a/output/nav_changes_2026-04-08.xlsx
+++ b/output/nav_changes_2026-04-08.xlsx
@@ -930,7 +930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2944,47 +2944,47 @@
           <t>2026-02-09</t>
         </is>
       </c>
-      <c r="B41" s="4" t="n">
-        <v>-0.004648</v>
-      </c>
-      <c r="C41" s="4" t="n">
-        <v>-0.003856</v>
-      </c>
-      <c r="D41" s="4" t="n">
-        <v>-0.003283</v>
-      </c>
-      <c r="E41" s="4" t="n">
-        <v>-0.003031</v>
-      </c>
-      <c r="F41" s="4" t="n">
-        <v>-0.008221000000000001</v>
+      <c r="B41" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>0.000318</v>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>0.001473</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>0.0004639999999999999</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0.000241</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>-0.020143</v>
-      </c>
-      <c r="H41" s="4" t="n">
-        <v>-0.000395</v>
+        <v>-0.004288</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>0.001668</v>
       </c>
       <c r="I41" s="4" t="n">
-        <v>-0.003991</v>
-      </c>
-      <c r="J41" s="4" t="n">
-        <v>-0.002995</v>
-      </c>
-      <c r="K41" s="4" t="n">
-        <v>-0.002604</v>
-      </c>
-      <c r="L41" s="4" t="n">
-        <v>-0.003112</v>
-      </c>
-      <c r="M41" s="4" t="n">
-        <v>-0.00127</v>
-      </c>
-      <c r="N41" s="4" t="n">
-        <v>-0.00177</v>
+        <v>-0.0005020000000000001</v>
+      </c>
+      <c r="J41" s="6" t="n">
+        <v>0.000489</v>
+      </c>
+      <c r="K41" s="6" t="n">
+        <v>0.001628</v>
+      </c>
+      <c r="L41" s="6" t="n">
+        <v>0.0006850000000000001</v>
+      </c>
+      <c r="M41" s="6" t="n">
+        <v>0.000163</v>
+      </c>
+      <c r="N41" s="6" t="n">
+        <v>0.000114</v>
       </c>
       <c r="O41" s="4" t="n">
-        <v>-0.007792</v>
+        <v>-0.000164</v>
       </c>
     </row>
     <row r="42">
@@ -2994,46 +2994,46 @@
         </is>
       </c>
       <c r="B42" s="6" t="n">
-        <v>0.000998</v>
+        <v>0.0009970000000000001</v>
       </c>
       <c r="C42" s="6" t="n">
-        <v>0.000396</v>
+        <v>0.000398</v>
       </c>
       <c r="D42" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>0.000458</v>
+        <v>0.000459</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>0.000513</v>
+        <v>0.0005099999999999999</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>-0.002038</v>
+        <v>-0.00204</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>0.005980999999999999</v>
+        <v>0.005979</v>
       </c>
       <c r="I42" s="6" t="n">
-        <v>0.000505</v>
+        <v>0.0005020000000000001</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>0.0009810000000000001</v>
+        <v>0.000985</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>0.001635</v>
+        <v>0.001636</v>
       </c>
       <c r="L42" s="6" t="n">
-        <v>0.000364</v>
+        <v>0.000365</v>
       </c>
       <c r="M42" s="6" t="n">
         <v>0.000511</v>
       </c>
       <c r="N42" s="6" t="n">
-        <v>0.000499</v>
+        <v>0.0005</v>
       </c>
       <c r="O42" s="6" t="n">
-        <v>0.000163</v>
+        <v>0.000164</v>
       </c>
     </row>
     <row r="43">
@@ -3043,10 +3043,10 @@
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>-0.001497</v>
+        <v>-0.001499</v>
       </c>
       <c r="C43" s="6" t="n">
-        <v>0.000339</v>
+        <v>0.000341</v>
       </c>
       <c r="D43" s="9" t="n">
         <v>0</v>
@@ -3055,34 +3055,34 @@
         <v>0.002772</v>
       </c>
       <c r="F43" s="6" t="n">
-        <v>0.000316</v>
+        <v>0.000319</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>-0.000879</v>
+        <v>-0.0008719999999999999</v>
       </c>
       <c r="H43" s="4" t="n">
-        <v>-0.008935999999999999</v>
+        <v>-0.008933999999999999</v>
       </c>
       <c r="I43" s="6" t="n">
-        <v>0.004555</v>
+        <v>0.004556</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>0.0004929999999999999</v>
+        <v>0.00049</v>
       </c>
       <c r="K43" s="6" t="n">
-        <v>0.000273</v>
+        <v>0.000275</v>
       </c>
       <c r="L43" s="6" t="n">
-        <v>0.0009229999999999999</v>
+        <v>0.0009270000000000001</v>
       </c>
       <c r="M43" s="6" t="n">
-        <v>0.00197</v>
+        <v>0.001962</v>
       </c>
       <c r="N43" s="6" t="n">
-        <v>0.0006469999999999999</v>
+        <v>0.0006489999999999999</v>
       </c>
       <c r="O43" s="6" t="n">
-        <v>0.001058</v>
+        <v>0.001066</v>
       </c>
     </row>
     <row r="44">
@@ -3095,43 +3095,43 @@
         <v>0.001002</v>
       </c>
       <c r="C44" s="6" t="n">
-        <v>0.000623</v>
+        <v>0.000625</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>0.000494</v>
+        <v>0.000491</v>
       </c>
       <c r="E44" s="4" t="n">
         <v>-0.001384</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>0.000183</v>
+        <v>0.000184</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>0.0006619999999999999</v>
       </c>
       <c r="H44" s="4" t="n">
-        <v>-0.001124</v>
+        <v>-0.001119</v>
       </c>
       <c r="I44" s="4" t="n">
-        <v>-0.001009</v>
+        <v>-0.001013</v>
       </c>
       <c r="J44" s="6" t="n">
-        <v>0.000494</v>
+        <v>0.00049</v>
       </c>
       <c r="K44" s="4" t="n">
-        <v>-0.000273</v>
+        <v>-0.000275</v>
       </c>
       <c r="L44" s="4" t="n">
-        <v>-0.00047</v>
+        <v>-0.000472</v>
       </c>
       <c r="M44" s="6" t="n">
         <v>4.400000000000001e-05</v>
       </c>
       <c r="N44" s="6" t="n">
-        <v>0.000432</v>
+        <v>0.000433</v>
       </c>
       <c r="O44" s="6" t="n">
-        <v>0.000122</v>
+        <v>0.000113</v>
       </c>
     </row>
     <row r="45">
@@ -3141,25 +3141,25 @@
         </is>
       </c>
       <c r="B45" s="4" t="n">
-        <v>-0.000501</v>
+        <v>-0.000498</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>0.00026</v>
+        <v>0.000262</v>
       </c>
       <c r="D45" s="4" t="n">
-        <v>-0.000494</v>
+        <v>-0.000491</v>
       </c>
       <c r="E45" s="9" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>-9.1e-05</v>
+        <v>-9.2e-05</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>0.0005899999999999999</v>
+        <v>0.000589</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>0.00392</v>
+        <v>0.003914</v>
       </c>
       <c r="I45" s="9" t="n">
         <v>0</v>
@@ -3168,19 +3168,19 @@
         <v>0</v>
       </c>
       <c r="K45" s="6" t="n">
-        <v>0.0008210000000000001</v>
+        <v>0.000819</v>
       </c>
       <c r="L45" s="6" t="n">
-        <v>0.000257</v>
+        <v>0.000258</v>
       </c>
       <c r="M45" s="4" t="n">
         <v>-1.1e-05</v>
       </c>
       <c r="N45" s="4" t="n">
-        <v>-0.000204</v>
+        <v>-0.000205</v>
       </c>
       <c r="O45" s="4" t="n">
-        <v>-0.000122</v>
+        <v>-0.000113</v>
       </c>
     </row>
     <row r="46">
@@ -3190,28 +3190,28 @@
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>0.000501</v>
+        <v>0.000498</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>0.000193</v>
+        <v>0.000182</v>
       </c>
       <c r="D46" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>-0.000463</v>
+        <v>-0.00046</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>-6.3e-05</v>
+        <v>-6.4e-05</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>8.3e-05</v>
+        <v>8.4e-05</v>
       </c>
       <c r="H46" s="6" t="n">
         <v>7e-06</v>
       </c>
       <c r="I46" s="4" t="n">
-        <v>-0.001014</v>
+        <v>-0.001007</v>
       </c>
       <c r="J46" s="9" t="n">
         <v>0</v>
@@ -3220,16 +3220,16 @@
         <v>-0.001361</v>
       </c>
       <c r="L46" s="6" t="n">
-        <v>0.001244</v>
+        <v>0.00124</v>
       </c>
       <c r="M46" s="4" t="n">
-        <v>-0.0009239999999999999</v>
+        <v>-0.000915</v>
       </c>
       <c r="N46" s="6" t="n">
-        <v>0.0005909999999999999</v>
+        <v>0.0005920000000000001</v>
       </c>
       <c r="O46" s="6" t="n">
-        <v>0.000376</v>
+        <v>0.000369</v>
       </c>
     </row>
     <row r="47">
@@ -3242,43 +3242,43 @@
         <v>0</v>
       </c>
       <c r="C47" s="6" t="n">
-        <v>0.000136</v>
+        <v>0.000148</v>
       </c>
       <c r="D47" s="9" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>0.0009260000000000001</v>
+        <v>0.00092</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>-0.000239</v>
+        <v>-0.000241</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>-0.001354</v>
+        <v>-0.001355</v>
       </c>
       <c r="H47" s="4" t="n">
-        <v>-0.011534</v>
+        <v>-0.01153</v>
       </c>
       <c r="I47" s="4" t="n">
-        <v>-0.000501</v>
+        <v>-0.000508</v>
       </c>
       <c r="J47" s="9" t="n">
         <v>0</v>
       </c>
       <c r="K47" s="4" t="n">
-        <v>-0.002176</v>
+        <v>-0.002174</v>
       </c>
       <c r="L47" s="4" t="n">
-        <v>-0.00079</v>
+        <v>-0.000784</v>
       </c>
       <c r="M47" s="4" t="n">
-        <v>-0.000619</v>
+        <v>-0.00062</v>
       </c>
       <c r="N47" s="4" t="n">
         <v>-0.000398</v>
       </c>
       <c r="O47" s="6" t="n">
-        <v>0.000428</v>
+        <v>0.000431</v>
       </c>
     </row>
     <row r="48">
@@ -3291,43 +3291,43 @@
         <v>0.000998</v>
       </c>
       <c r="C48" s="6" t="n">
-        <v>6.8e-05</v>
+        <v>5.7e-05</v>
       </c>
       <c r="D48" s="6" t="n">
         <v>0.0009829999999999999</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>0.0009220000000000001</v>
+        <v>0.0009260000000000001</v>
       </c>
       <c r="F48" s="6" t="n">
-        <v>0.000309</v>
+        <v>0.000312</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>-0.000548</v>
+        <v>-0.000546</v>
       </c>
       <c r="H48" s="4" t="n">
-        <v>-0.002343</v>
+        <v>-0.002341</v>
       </c>
       <c r="I48" s="6" t="n">
-        <v>0.0005020000000000001</v>
+        <v>0.000509</v>
       </c>
       <c r="J48" s="6" t="n">
-        <v>0.0009829999999999999</v>
+        <v>0.000987</v>
       </c>
       <c r="K48" s="6" t="n">
-        <v>0.001633</v>
+        <v>0.001635</v>
       </c>
       <c r="L48" s="4" t="n">
-        <v>-0.000337</v>
+        <v>-0.000339</v>
       </c>
       <c r="M48" s="6" t="n">
         <v>0.000555</v>
       </c>
       <c r="N48" s="4" t="n">
-        <v>-0.000136</v>
+        <v>-0.000137</v>
       </c>
       <c r="O48" s="4" t="n">
-        <v>-0.000204</v>
+        <v>-0.000205</v>
       </c>
     </row>
     <row r="49">
@@ -3343,40 +3343,40 @@
         <v>0.000159</v>
       </c>
       <c r="D49" s="6" t="n">
-        <v>0.000494</v>
+        <v>0.000492</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>0.0004639999999999999</v>
+        <v>0.000461</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>-4.9e-05</v>
+        <v>-5e-05</v>
       </c>
       <c r="G49" s="6" t="n">
-        <v>0.000837</v>
+        <v>0.00083</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>0.002943</v>
+        <v>0.002935</v>
       </c>
       <c r="I49" s="4" t="n">
         <v>-0.001513</v>
       </c>
       <c r="J49" s="6" t="n">
-        <v>0.000494</v>
+        <v>0.000491</v>
       </c>
       <c r="K49" s="6" t="n">
-        <v>0.002184</v>
+        <v>0.002182</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>-0.000497</v>
+        <v>-0.000499</v>
       </c>
       <c r="M49" s="4" t="n">
         <v>-2.2e-05</v>
       </c>
       <c r="N49" s="4" t="n">
-        <v>-0.00101</v>
+        <v>-0.001012</v>
       </c>
       <c r="O49" s="4" t="n">
-        <v>-0.000285</v>
+        <v>-0.000287</v>
       </c>
     </row>
     <row r="50">
@@ -3386,43 +3386,43 @@
         </is>
       </c>
       <c r="B50" s="6" t="n">
-        <v>0.000452</v>
+        <v>0.000454</v>
       </c>
       <c r="C50" s="6" t="n">
-        <v>0.000317</v>
+        <v>0.000319</v>
       </c>
       <c r="D50" s="4" t="n">
-        <v>-0.00123</v>
+        <v>-0.001231</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>0.000232</v>
+        <v>0.000233</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>-0.00073</v>
+        <v>-0.000729</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>-0.000992</v>
+        <v>-0.000987</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>0.000153</v>
+        <v>0.000161</v>
       </c>
       <c r="I50" s="4" t="n">
-        <v>-0.002111</v>
+        <v>-0.002113</v>
       </c>
       <c r="J50" s="4" t="n">
-        <v>-0.001968</v>
+        <v>-0.001965</v>
       </c>
       <c r="K50" s="4" t="n">
-        <v>-0.002179</v>
+        <v>-0.002178</v>
       </c>
       <c r="L50" s="4" t="n">
-        <v>-0.001072</v>
+        <v>-0.001076</v>
       </c>
       <c r="M50" s="4" t="n">
-        <v>-0.000739</v>
+        <v>-0.00074</v>
       </c>
       <c r="N50" s="4" t="n">
-        <v>-0.0009180000000000001</v>
+        <v>-0.00092</v>
       </c>
       <c r="O50" s="4" t="n">
         <v>-0.00126</v>
@@ -3435,46 +3435,46 @@
         </is>
       </c>
       <c r="B51" s="6" t="n">
-        <v>0.000497</v>
+        <v>0.000499</v>
       </c>
       <c r="C51" s="6" t="n">
-        <v>0.001158</v>
+        <v>0.001162</v>
       </c>
       <c r="D51" s="6" t="n">
-        <v>0.0009790000000000001</v>
+        <v>0.0009829999999999999</v>
       </c>
       <c r="E51" s="9" t="n">
         <v>0</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>0.00197</v>
+        <v>0.001965</v>
       </c>
       <c r="G51" s="6" t="n">
-        <v>0.000207</v>
+        <v>0.00021</v>
       </c>
       <c r="H51" s="6" t="n">
-        <v>0.004125</v>
+        <v>0.004119</v>
       </c>
       <c r="I51" s="6" t="n">
-        <v>0.001001</v>
+        <v>0.001004</v>
       </c>
       <c r="J51" s="6" t="n">
         <v>0.002949</v>
       </c>
       <c r="K51" s="6" t="n">
-        <v>0.001088</v>
+        <v>0.001087</v>
       </c>
       <c r="L51" s="6" t="n">
-        <v>0.001696</v>
+        <v>0.001702</v>
       </c>
       <c r="M51" s="6" t="n">
-        <v>0.001949</v>
+        <v>0.00194</v>
       </c>
       <c r="N51" s="6" t="n">
-        <v>0.001067</v>
+        <v>0.001069</v>
       </c>
       <c r="O51" s="6" t="n">
-        <v>0.001822</v>
+        <v>0.001826</v>
       </c>
     </row>
     <row r="52">
@@ -3484,46 +3484,46 @@
         </is>
       </c>
       <c r="B52" s="6" t="n">
-        <v>0.0005020000000000001</v>
+        <v>0.0005</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>-0.000272</v>
+        <v>-0.000273</v>
       </c>
       <c r="D52" s="6" t="n">
         <v>0.001961</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>0.000459</v>
+        <v>0.000461</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>-0.00038</v>
+        <v>-0.000376</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>-0.000341</v>
+        <v>-0.000346</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>0.0007149999999999999</v>
+        <v>0.0007159999999999999</v>
       </c>
       <c r="I52" s="6" t="n">
-        <v>0.0005059999999999999</v>
+        <v>0.0005020000000000001</v>
       </c>
       <c r="J52" s="4" t="n">
-        <v>-0.000495</v>
+        <v>-0.000491</v>
       </c>
       <c r="K52" s="6" t="n">
-        <v>0.001912</v>
+        <v>0.001909</v>
       </c>
       <c r="L52" s="4" t="n">
-        <v>-0.000719</v>
+        <v>-0.000721</v>
       </c>
       <c r="M52" s="6" t="n">
         <v>0.000414</v>
       </c>
       <c r="N52" s="4" t="n">
-        <v>-0.000556</v>
+        <v>-0.000557</v>
       </c>
       <c r="O52" s="4" t="n">
-        <v>-0.000326</v>
+        <v>-0.000328</v>
       </c>
     </row>
     <row r="53">
@@ -3536,25 +3536,25 @@
         <v>0</v>
       </c>
       <c r="C53" s="6" t="n">
-        <v>0.000931</v>
+        <v>0.000935</v>
       </c>
       <c r="D53" s="6" t="n">
-        <v>0.000982</v>
+        <v>0.0009810000000000001</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>0.002307</v>
+        <v>0.00231</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>0.001437</v>
+        <v>0.001435</v>
       </c>
       <c r="G53" s="6" t="n">
-        <v>0.001137</v>
+        <v>0.001135</v>
       </c>
       <c r="H53" s="6" t="n">
-        <v>0.005277</v>
+        <v>0.005274</v>
       </c>
       <c r="I53" s="6" t="n">
-        <v>0.002012</v>
+        <v>0.002009</v>
       </c>
       <c r="J53" s="6" t="n">
         <v>0.001476</v>
@@ -3563,16 +3563,16 @@
         <v>0.002521</v>
       </c>
       <c r="L53" s="6" t="n">
-        <v>0.001493</v>
+        <v>0.001489</v>
       </c>
       <c r="M53" s="6" t="n">
-        <v>0.001167</v>
+        <v>0.001168</v>
       </c>
       <c r="N53" s="6" t="n">
-        <v>0.00067</v>
+        <v>0.000671</v>
       </c>
       <c r="O53" s="6" t="n">
-        <v>0.000896</v>
+        <v>0.000893</v>
       </c>
     </row>
     <row r="54">
@@ -3582,28 +3582,28 @@
         </is>
       </c>
       <c r="B54" s="6" t="n">
-        <v>0.000498</v>
+        <v>0.000495</v>
       </c>
       <c r="C54" s="6" t="n">
-        <v>0.0007729999999999999</v>
+        <v>0.0007649999999999999</v>
       </c>
       <c r="D54" s="4" t="n">
-        <v>-0.000491</v>
+        <v>-0.000488</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>-0.00046</v>
+        <v>-0.000462</v>
       </c>
       <c r="F54" s="6" t="n">
-        <v>0.00067</v>
+        <v>0.000668</v>
       </c>
       <c r="G54" s="6" t="n">
-        <v>0.000569</v>
+        <v>0.000568</v>
       </c>
       <c r="H54" s="6" t="n">
-        <v>0.003095</v>
+        <v>0.003102</v>
       </c>
       <c r="I54" s="6" t="n">
-        <v>0.006077</v>
+        <v>0.006078</v>
       </c>
       <c r="J54" s="6" t="n">
         <v>0.001478</v>
@@ -3612,13 +3612,13 @@
         <v>-0.003813</v>
       </c>
       <c r="L54" s="6" t="n">
-        <v>0.001067</v>
+        <v>0.001071</v>
       </c>
       <c r="M54" s="6" t="n">
-        <v>0.002229</v>
+        <v>0.002232</v>
       </c>
       <c r="N54" s="6" t="n">
-        <v>0.00166</v>
+        <v>0.001663</v>
       </c>
       <c r="O54" s="6" t="n">
         <v>0.001336</v>
@@ -3631,44 +3631,44 @@
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>-0.001496</v>
+        <v>-0.001492</v>
       </c>
       <c r="C55" s="4" t="n">
-        <v>-0.0007040000000000001</v>
+        <v>-0.000696</v>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" s="6" t="n">
-        <v>0.00046</v>
+        <v>0.000462</v>
       </c>
       <c r="F55" s="4" t="n">
         <v>-0.001632</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>-0.001745</v>
+        <v>-0.001742</v>
       </c>
       <c r="H55" s="6" t="n">
-        <v>0.000438</v>
+        <v>0.000432</v>
       </c>
       <c r="I55" s="4" t="n">
-        <v>-0.012007</v>
+        <v>-0.012004</v>
       </c>
       <c r="J55" s="4" t="n">
-        <v>-0.001965</v>
+        <v>-0.001967</v>
       </c>
       <c r="K55" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L55" s="4" t="n">
-        <v>-0.002555</v>
+        <v>-0.002556</v>
       </c>
       <c r="M55" s="4" t="n">
-        <v>-0.003853</v>
+        <v>-0.003859</v>
       </c>
       <c r="N55" s="4" t="n">
-        <v>-0.002642</v>
+        <v>-0.002647</v>
       </c>
       <c r="O55" s="4" t="n">
-        <v>-0.002249</v>
+        <v>-0.002246</v>
       </c>
     </row>
     <row r="56">
@@ -3681,41 +3681,41 @@
         <v>0</v>
       </c>
       <c r="C56" s="6" t="n">
-        <v>0.000329</v>
+        <v>0.000331</v>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" s="4" t="n">
-        <v>-0.001379</v>
+        <v>-0.001384</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>-0.000295</v>
+        <v>-0.000291</v>
       </c>
       <c r="G56" s="6" t="n">
-        <v>0.000527</v>
+        <v>0.000525</v>
       </c>
       <c r="H56" s="6" t="n">
-        <v>0.000906</v>
+        <v>0.0009080000000000001</v>
       </c>
       <c r="I56" s="6" t="n">
-        <v>0.005536</v>
+        <v>0.00553</v>
       </c>
       <c r="J56" s="4" t="n">
-        <v>-0.0009840000000000001</v>
+        <v>-0.0009829999999999999</v>
       </c>
       <c r="K56" s="4" t="n">
         <v>-0.002712</v>
       </c>
       <c r="L56" s="4" t="n">
-        <v>-0.000355</v>
+        <v>-0.000356</v>
       </c>
       <c r="M56" s="4" t="n">
-        <v>-0.001066</v>
+        <v>-0.001056</v>
       </c>
       <c r="N56" s="4" t="n">
-        <v>-0.000215</v>
+        <v>-0.000216</v>
       </c>
       <c r="O56" s="4" t="n">
-        <v>-0.000478</v>
+        <v>-0.000482</v>
       </c>
     </row>
     <row r="57">
@@ -3727,40 +3727,42 @@
       <c r="B57" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" s="6" t="n">
+        <v>0.000148</v>
+      </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" s="4" t="n">
-        <v>-0.0004639999999999999</v>
+        <v>-0.000461</v>
       </c>
       <c r="F57" s="4" t="n">
         <v>-0.000787</v>
       </c>
       <c r="G57" s="6" t="n">
-        <v>0.000724</v>
+        <v>0.000725</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>-0.001343</v>
+        <v>-0.001338</v>
       </c>
       <c r="I57" s="4" t="n">
-        <v>-0.002511</v>
+        <v>-0.002504</v>
       </c>
       <c r="J57" s="4" t="n">
-        <v>-0.0009779999999999999</v>
+        <v>-0.000982</v>
       </c>
       <c r="K57" s="6" t="n">
-        <v>0.002176</v>
+        <v>0.002175</v>
       </c>
       <c r="L57" s="4" t="n">
-        <v>-0.0006469999999999999</v>
+        <v>-0.0006489999999999999</v>
       </c>
       <c r="M57" s="4" t="n">
-        <v>-0.001542</v>
+        <v>-0.001544</v>
       </c>
       <c r="N57" s="4" t="n">
-        <v>-0.001268</v>
+        <v>-0.001259</v>
       </c>
       <c r="O57" s="4" t="n">
-        <v>-0.000661</v>
+        <v>-0.000656</v>
       </c>
     </row>
     <row r="58">
@@ -3770,42 +3772,44 @@
         </is>
       </c>
       <c r="B58" s="6" t="n">
-        <v>0.000497</v>
-      </c>
-      <c r="C58" t="inlineStr"/>
+        <v>0.000499</v>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>0.000331</v>
+      </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" s="6" t="n">
-        <v>0.000925</v>
+        <v>0.0009229999999999999</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>0.000746</v>
+        <v>0.000745</v>
       </c>
       <c r="G58" s="6" t="n">
-        <v>0.000724</v>
+        <v>0.000726</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>0.000467</v>
+        <v>0.000461</v>
       </c>
       <c r="I58" s="4" t="n">
         <v>-0.001503</v>
       </c>
       <c r="J58" s="6" t="n">
-        <v>0.002457</v>
+        <v>0.00246</v>
       </c>
       <c r="K58" s="4" t="n">
-        <v>-0.001632</v>
+        <v>-0.001628</v>
       </c>
       <c r="L58" s="6" t="n">
-        <v>0.00023</v>
+        <v>0.000231</v>
       </c>
       <c r="M58" s="4" t="n">
         <v>-0.000293</v>
       </c>
       <c r="N58" s="6" t="n">
-        <v>0.00026</v>
+        <v>0.000261</v>
       </c>
       <c r="O58" s="6" t="n">
-        <v>0.00057</v>
+        <v>0.000574</v>
       </c>
     </row>
     <row r="59">
@@ -3815,39 +3819,41 @@
         </is>
       </c>
       <c r="B59" s="6" t="n">
-        <v>0.0005020000000000001</v>
-      </c>
-      <c r="C59" t="inlineStr"/>
+        <v>0.0005</v>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>0.000354</v>
+      </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" s="6" t="n">
-        <v>0.00231</v>
+        <v>0.002309</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>0.001465</v>
+        <v>0.001463</v>
       </c>
       <c r="G59" s="6" t="n">
-        <v>0.000311</v>
+        <v>0.000316</v>
       </c>
       <c r="H59" s="6" t="n">
-        <v>0.001147</v>
+        <v>0.001156</v>
       </c>
       <c r="I59" s="6" t="n">
-        <v>0.002513</v>
+        <v>0.002512</v>
       </c>
       <c r="J59" s="6" t="n">
-        <v>0.001975</v>
+        <v>0.001972</v>
       </c>
       <c r="K59" s="6" t="n">
-        <v>0.000546</v>
+        <v>0.000543</v>
       </c>
       <c r="L59" s="6" t="n">
-        <v>0.0007630000000000001</v>
+        <v>0.000766</v>
       </c>
       <c r="M59" s="6" t="n">
-        <v>0.001337</v>
+        <v>0.001339</v>
       </c>
       <c r="N59" s="6" t="n">
-        <v>0.0016</v>
+        <v>0.001591</v>
       </c>
       <c r="O59" s="6" t="n">
         <v>0.001375</v>
@@ -3862,40 +3868,324 @@
       <c r="B60" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" s="4" t="n">
+        <v>-0.000616</v>
+      </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" s="4" t="n">
-        <v>-0.000461</v>
+        <v>-0.000458</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>5.6e-05</v>
+        <v>5.7e-05</v>
       </c>
       <c r="G60" s="6" t="n">
-        <v>0.000964</v>
+        <v>0.000958</v>
       </c>
       <c r="H60" s="6" t="n">
-        <v>0.000552</v>
+        <v>0.000546</v>
       </c>
       <c r="I60" s="6" t="n">
-        <v>0.002515</v>
+        <v>0.002513</v>
       </c>
       <c r="J60" s="4" t="n">
-        <v>-0.000496</v>
+        <v>-0.0004929999999999999</v>
       </c>
       <c r="K60" s="6" t="n">
-        <v>0.002997</v>
+        <v>0.002999</v>
       </c>
       <c r="L60" s="6" t="n">
-        <v>0.000319</v>
+        <v>0.000312</v>
       </c>
       <c r="M60" s="4" t="n">
-        <v>-0.000684</v>
+        <v>-0.0006850000000000001</v>
       </c>
       <c r="N60" s="6" t="n">
-        <v>0.000942</v>
+        <v>0.000956</v>
       </c>
       <c r="O60" s="9" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="n">
+        <v>0.000495</v>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>0.0009940000000000001</v>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" s="4" t="n">
+        <v>-0.000462</v>
+      </c>
+      <c r="F61" s="4" t="n">
+        <v>-0.000242</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>0.0007689999999999999</v>
+      </c>
+      <c r="H61" s="6" t="n">
+        <v>0.002305</v>
+      </c>
+      <c r="I61" s="4" t="n">
+        <v>-0.002011</v>
+      </c>
+      <c r="J61" s="4" t="n">
+        <v>-0.0004929999999999999</v>
+      </c>
+      <c r="K61" s="4" t="n">
+        <v>-0.000544</v>
+      </c>
+      <c r="L61" s="4" t="n">
+        <v>-0.000116</v>
+      </c>
+      <c r="M61" s="6" t="n">
+        <v>0.000163</v>
+      </c>
+      <c r="N61" s="4" t="n">
+        <v>-0.000523</v>
+      </c>
+      <c r="O61" s="4" t="n">
+        <v>-0.000318</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>0.000366</v>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" s="6" t="n">
+        <v>0.002312</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>0.001302</v>
+      </c>
+      <c r="G62" s="6" t="n">
+        <v>0.000696</v>
+      </c>
+      <c r="H62" s="6" t="n">
+        <v>0.001396</v>
+      </c>
+      <c r="I62" s="6" t="n">
+        <v>0.003531</v>
+      </c>
+      <c r="J62" s="6" t="n">
+        <v>0.00148</v>
+      </c>
+      <c r="K62" s="6" t="n">
+        <v>0.000275</v>
+      </c>
+      <c r="L62" s="6" t="n">
+        <v>0.001302</v>
+      </c>
+      <c r="M62" s="6" t="n">
+        <v>0.00086</v>
+      </c>
+      <c r="N62" s="6" t="n">
+        <v>0.001332</v>
+      </c>
+      <c r="O62" s="6" t="n">
+        <v>0.001243</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="n">
+        <v>-0.001493</v>
+      </c>
+      <c r="C63" s="6" t="n">
+        <v>0.000126</v>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" s="4" t="n">
+        <v>-0.001388</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>-4.3e-05</v>
+      </c>
+      <c r="G63" s="6" t="n">
+        <v>0.000127</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>-0.000434</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>-0.003017</v>
+      </c>
+      <c r="J63" s="6" t="n">
+        <v>0.0004929999999999999</v>
+      </c>
+      <c r="K63" s="4" t="n">
+        <v>-0.001093</v>
+      </c>
+      <c r="L63" s="4" t="n">
+        <v>-7.1e-05</v>
+      </c>
+      <c r="M63" s="4" t="n">
+        <v>-0.000957</v>
+      </c>
+      <c r="N63" s="4" t="n">
+        <v>-0.001296</v>
+      </c>
+      <c r="O63" s="4" t="n">
+        <v>-0.0006980000000000001</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="n">
+        <v>0.000995</v>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>0.000354</v>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" s="6" t="n">
+        <v>0.0009260000000000001</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>0.001831</v>
+      </c>
+      <c r="G64" s="6" t="n">
+        <v>0.000728</v>
+      </c>
+      <c r="H64" s="6" t="n">
+        <v>0.001433</v>
+      </c>
+      <c r="I64" s="6" t="n">
+        <v>0.001511</v>
+      </c>
+      <c r="J64" s="6" t="n">
+        <v>0.001978</v>
+      </c>
+      <c r="K64" s="6" t="n">
+        <v>0.00055</v>
+      </c>
+      <c r="L64" s="6" t="n">
+        <v>0.0009909999999999999</v>
+      </c>
+      <c r="M64" s="6" t="n">
+        <v>0.001547</v>
+      </c>
+      <c r="N64" s="6" t="n">
+        <v>0.001686</v>
+      </c>
+      <c r="O64" s="6" t="n">
+        <v>0.001635</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="n">
+        <v>0.001001</v>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>0.000538</v>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" s="6" t="n">
+        <v>0.000463</v>
+      </c>
+      <c r="F65" s="4" t="n">
+        <v>-7.8e-05</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <v>0.001162</v>
+      </c>
+      <c r="H65" s="6" t="n">
+        <v>0.004599</v>
+      </c>
+      <c r="I65" s="4" t="n">
+        <v>-0.000503</v>
+      </c>
+      <c r="J65" s="4" t="n">
+        <v>-0.000494</v>
+      </c>
+      <c r="K65" s="6" t="n">
+        <v>0.001635</v>
+      </c>
+      <c r="L65" s="6" t="n">
+        <v>0.001627</v>
+      </c>
+      <c r="M65" s="6" t="n">
+        <v>0.000381</v>
+      </c>
+      <c r="N65" s="6" t="n">
+        <v>0.000273</v>
+      </c>
+      <c r="O65" s="6" t="n">
+        <v>0.000247</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>0.000973</v>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" s="6" t="n">
+        <v>0.00372</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>0.00245</v>
+      </c>
+      <c r="G66" s="6" t="n">
+        <v>0.000211</v>
+      </c>
+      <c r="H66" s="6" t="n">
+        <v>0.00327</v>
+      </c>
+      <c r="I66" s="6" t="n">
+        <v>0.002523</v>
+      </c>
+      <c r="J66" s="6" t="n">
+        <v>0.002477</v>
+      </c>
+      <c r="K66" s="6" t="n">
+        <v>0.001091</v>
+      </c>
+      <c r="L66" s="6" t="n">
+        <v>0.001585</v>
+      </c>
+      <c r="M66" s="6" t="n">
+        <v>0.001353</v>
+      </c>
+      <c r="N66" s="6" t="n">
+        <v>0.001472</v>
+      </c>
+      <c r="O66" s="6" t="n">
+        <v>0.002041</v>
       </c>
     </row>
   </sheetData>

</xml_diff>